<commit_message>
feat: udvid garnkatalog og FAQ
Tilføjer FAQ-indhold og side, opdaterer garnkatalogets import/Excel-flow og udvider katalog-integration (farver, barcode, substitution-forbedringer).

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/STRIQ_ideer.xlsx
+++ b/STRIQ_ideer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\AI_projects\maskerummet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA3F5AA5-7884-475C-8250-D8C965267645}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27629910-090C-4043-BD9D-4C7F6A450A40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10" yWindow="10" windowWidth="24940" windowHeight="15900" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10" yWindow="10" windowWidth="24940" windowHeight="15900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="STRIQ Ideer" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="Garnforhandlernes websites" sheetId="3" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'STRIQ Ideer'!$A$1:$D$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'STRIQ Ideer'!$A$1:$D$43</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="123">
   <si>
     <t>Kategori</t>
   </si>
@@ -55,15 +55,6 @@
     <t>Garnlager</t>
   </si>
   <si>
-    <t>Import fra Ravelry</t>
-  </si>
-  <si>
-    <t>API eller CSV export fra hkwermuth-profilen</t>
-  </si>
-  <si>
-    <t>Garnsubstitution baseret på stash</t>
-  </si>
-  <si>
     <t>Fiber-kategorier til filter</t>
   </si>
   <si>
@@ -71,15 +62,6 @@
   </si>
   <si>
     <t>Metrage-beregner pr. projekt</t>
-  </si>
-  <si>
-    <t>Svært at slette i dette men skal kunne redigere</t>
-  </si>
-  <si>
-    <t>Strikkefasthed</t>
-  </si>
-  <si>
-    <t>Strikkefasthed skal tilføjes</t>
   </si>
   <si>
     <t>Man skal kunne sortere i garnlagere</t>
@@ -240,9 +222,6 @@
   </si>
   <si>
     <t>Spørgekasse</t>
-  </si>
-  <si>
-    <t>Hvordan undgår man at garn fnulrer</t>
   </si>
   <si>
     <t>Trænet AI-mønstergenkendelse</t>
@@ -607,6 +586,72 @@
   </si>
   <si>
     <t>KnittingforOlive.dk, sandnesgarn.dk, www.garnstudio.com, hjertegarn.dk og isagerstrik.dk</t>
+  </si>
+  <si>
+    <t>Markere garn man selv har</t>
+  </si>
+  <si>
+    <t>Man skal kunne angive hvilke(n) farve(r) man har garnet i. Skal være muligt kun at søge i de garner man selv har</t>
+  </si>
+  <si>
+    <t>Ønskeliste med garner</t>
+  </si>
+  <si>
+    <t>Man skal kunne lave en liste over garner / farver man synes ser spændende ud</t>
+  </si>
+  <si>
+    <t>Fotos af alle garner - skal det ligge i garn-kataloget og vælges når man laver sit eget garnlager eller uploades individuelt. Tænker at mulighed for at vælge skal være der, men default får man den fra garnkataloget</t>
+  </si>
+  <si>
+    <t>Farveteori implementeret ift. egne garner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hvrodan skal min næste sweater se ud, hvor man bruger sine egne garner, evt. vælger at man vil købe ekstra i en bestemt farve og så for man forslag ud fra om man ønsker en top, bluse, sweater osv. Og vælger om det skal være en varm/kølig osv. </t>
+  </si>
+  <si>
+    <t>certificeringer</t>
+  </si>
+  <si>
+    <t>Hvad betyder de forskellige typer certificeringer, fx GOTS, øketex osv</t>
+  </si>
+  <si>
+    <t>Fingering, Lace osv</t>
+  </si>
+  <si>
+    <t>Forklaring til ordene og så skal det være mere mundrette ord som alle forstår der vises i databasen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brugervenlighed af databasen. </t>
+  </si>
+  <si>
+    <t>Kan jeg lave en gennemgang med virtuelle testpersoner?</t>
+  </si>
+  <si>
+    <t>Fotos af alle garner i databasen</t>
+  </si>
+  <si>
+    <t>Hvad vil det kræve/fylde. Hvor mange garner findes</t>
+  </si>
+  <si>
+    <t>Man skal kunne skrive sin egne kommentarer</t>
+  </si>
+  <si>
+    <t>Garn man ønsker sig</t>
+  </si>
+  <si>
+    <t>Klikke rundt i garn og sætte dem på en ønskeliste. Evt. samarbejde med Ønskeskyen</t>
+  </si>
+  <si>
+    <t>garn</t>
+  </si>
+  <si>
+    <t>Udskydes indtil videre</t>
+  </si>
+  <si>
+    <t>Samle alle de steder jeg ønsker at opsnappe information fra i et LLM til garnspørgsmål</t>
+  </si>
+  <si>
+    <t>Hvordan undgår man at garn fnulrer. Hvad er de mest almindelige spørgsmål og svar på dem</t>
   </si>
 </sst>
 </file>
@@ -629,15 +674,18 @@
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -784,9 +832,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -800,6 +845,9 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1102,12 +1150,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D51"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="60" customWidth="1"/>
+    <col min="3" max="3" width="82.7265625" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1141,12 +1189,8 @@
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>6</v>
-      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="4"/>
       <c r="D4" s="5">
         <v>46101</v>
       </c>
@@ -1155,9 +1199,7 @@
       <c r="A5" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="B5" s="3"/>
       <c r="C5" s="4"/>
       <c r="D5" s="5">
         <v>46101</v>
@@ -1168,10 +1210,10 @@
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D6" s="5">
         <v>46101</v>
@@ -1182,7 +1224,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C7" s="4"/>
       <c r="D7" s="5">
@@ -1193,9 +1235,7 @@
       <c r="A8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>11</v>
-      </c>
+      <c r="B8" s="3"/>
       <c r="C8" s="4"/>
       <c r="D8" s="5">
         <v>46101</v>
@@ -1205,12 +1245,8 @@
       <c r="A9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="4"/>
       <c r="D9" s="5">
         <v>46101</v>
       </c>
@@ -1220,10 +1256,10 @@
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="D10" s="5">
         <v>46104</v>
@@ -1234,22 +1270,24 @@
         <v>4</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="4"/>
+        <v>10</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>116</v>
+      </c>
       <c r="D11" s="5">
         <v>46101</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="25">
+    <row r="12" spans="1:4" ht="17" customHeight="1">
       <c r="A12" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D12" s="5">
         <v>46104</v>
@@ -1260,10 +1298,10 @@
         <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D13" s="5">
         <v>46107</v>
@@ -1271,13 +1309,13 @@
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="D14" s="5">
         <v>46101</v>
@@ -1285,10 +1323,10 @@
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C15" s="4"/>
       <c r="D15" s="5">
@@ -1297,13 +1335,13 @@
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="D16" s="5">
         <v>46101</v>
@@ -1311,13 +1349,13 @@
     </row>
     <row r="17" spans="1:4" ht="25">
       <c r="A17" s="6" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="D17" s="5">
         <v>46101</v>
@@ -1325,13 +1363,13 @@
     </row>
     <row r="18" spans="1:4" ht="37.5">
       <c r="A18" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D18" s="5">
         <v>46101</v>
@@ -1339,13 +1377,13 @@
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D19" s="5">
         <v>46101</v>
@@ -1353,13 +1391,13 @@
     </row>
     <row r="20" spans="1:4" ht="25">
       <c r="A20" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="D20" s="5">
         <v>46101</v>
@@ -1367,13 +1405,13 @@
     </row>
     <row r="21" spans="1:4" ht="25">
       <c r="A21" s="6" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D21" s="5">
         <v>46104</v>
@@ -1381,64 +1419,66 @@
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="6" t="s">
-        <v>21</v>
+        <v>119</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>37</v>
+        <v>117</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>38</v>
+        <v>118</v>
       </c>
       <c r="D22" s="5">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" s="5">
         <v>46104</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="37.5">
-      <c r="A23" s="6" t="s">
+    <row r="24" spans="1:4" ht="37.5">
+      <c r="A24" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B23" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D23" s="5">
+      <c r="B24" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="5">
         <v>46111</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D24" s="5">
-        <v>46101</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C25" s="4"/>
+        <v>36</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="D25" s="5">
         <v>46101</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="7" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="5">
@@ -1447,39 +1487,39 @@
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="7" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>47</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="C27" s="4"/>
       <c r="D27" s="5">
         <v>46101</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="7" t="s">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C28" s="4"/>
+        <v>40</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="D28" s="5">
         <v>46101</v>
       </c>
     </row>
     <row r="29" spans="1:4">
-      <c r="A29" s="8" t="s">
-        <v>49</v>
+      <c r="A29" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>51</v>
+        <v>120</v>
       </c>
       <c r="D29" s="5">
         <v>46101</v>
@@ -1487,25 +1527,27 @@
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C30" s="4"/>
+        <v>44</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>45</v>
+      </c>
       <c r="D30" s="5">
         <v>46101</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>54</v>
+        <v>121</v>
       </c>
       <c r="D31" s="5">
         <v>46101</v>
@@ -1513,13 +1555,13 @@
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="8" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="D32" s="5">
         <v>46101</v>
@@ -1527,39 +1569,39 @@
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="B33" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B33" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C33" s="4"/>
+      <c r="C33" s="4" t="s">
+        <v>50</v>
+      </c>
       <c r="D33" s="5">
         <v>46101</v>
       </c>
     </row>
     <row r="34" spans="1:4">
-      <c r="A34" s="9" t="s">
-        <v>58</v>
+      <c r="A34" s="8" t="s">
+        <v>43</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>60</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="C34" s="4"/>
       <c r="D34" s="5">
         <v>46101</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="9" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="D35" s="5">
         <v>46101</v>
@@ -1567,115 +1609,118 @@
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="9" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C36" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>56</v>
+      </c>
       <c r="D36" s="5">
         <v>46101</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="9" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C37" s="4" t="s">
-        <v>65</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="C37" s="4"/>
       <c r="D37" s="5">
-        <v>46111</v>
+        <v>46101</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="9" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="D38" s="5">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D39" s="5">
         <v>46112</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="37.5">
-      <c r="A39" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D39" s="5">
+    <row r="40" spans="1:4" ht="37.5">
+      <c r="A40" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D40" s="5">
         <v>46120</v>
       </c>
     </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C40" s="4"/>
-      <c r="D40" s="5">
-        <v>46115</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="25">
+    <row r="41" spans="1:4">
       <c r="A41" s="9" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>70</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="C41" s="4"/>
       <c r="D41" s="5">
         <v>46115</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="25">
       <c r="A42" s="9" t="s">
-        <v>21</v>
+        <v>43</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>71</v>
+        <v>62</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="D42" s="5">
+        <v>46115</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="25">
+      <c r="A43" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D43" s="5">
         <v>46116</v>
       </c>
     </row>
-    <row r="43" spans="1:4" ht="26">
-      <c r="A43" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B43" s="10" t="s">
-        <v>73</v>
-      </c>
-      <c r="D43" s="12">
-        <v>46120</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4">
+    <row r="44" spans="1:4" ht="26">
       <c r="A44" s="11" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D44" s="12">
         <v>46120</v>
@@ -1683,10 +1728,10 @@
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="11" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B45" s="10" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="D45" s="12">
         <v>46120</v>
@@ -1694,10 +1739,10 @@
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="11" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B46" s="10" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="D46" s="12">
         <v>46120</v>
@@ -1705,13 +1750,10 @@
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="11" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B47" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="C47" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="D47" s="12">
         <v>46120</v>
@@ -1719,13 +1761,13 @@
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="11" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="C48" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D48" s="12">
         <v>46120</v>
@@ -1733,13 +1775,13 @@
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="11" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>82</v>
+        <v>72</v>
       </c>
       <c r="C49" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="D49" s="12">
         <v>46120</v>
@@ -1747,31 +1789,133 @@
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="11" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="C50" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="D50" s="12">
         <v>46120</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="26">
+    <row r="51" spans="1:4">
       <c r="A51" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="B51" s="13" t="s">
-        <v>87</v>
+        <v>78</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C51" t="s">
+        <v>77</v>
       </c>
       <c r="D51" s="12">
         <v>46120</v>
       </c>
     </row>
+    <row r="52" spans="1:4" ht="26">
+      <c r="A52" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D52" s="12">
+        <v>46120</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4">
+      <c r="A53" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B53" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="C53" t="s">
+        <v>102</v>
+      </c>
+      <c r="D53" s="12">
+        <v>46121</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4">
+      <c r="B57" t="s">
+        <v>103</v>
+      </c>
+      <c r="C57" t="s">
+        <v>104</v>
+      </c>
+      <c r="D57" s="12">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4">
+      <c r="B59" t="s">
+        <v>105</v>
+      </c>
+      <c r="D59" s="12">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="B60" t="s">
+        <v>106</v>
+      </c>
+      <c r="C60" t="s">
+        <v>107</v>
+      </c>
+      <c r="D60" s="12">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="B61" t="s">
+        <v>108</v>
+      </c>
+      <c r="C61" t="s">
+        <v>109</v>
+      </c>
+      <c r="D61" s="12">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="B62" t="s">
+        <v>110</v>
+      </c>
+      <c r="C62" t="s">
+        <v>111</v>
+      </c>
+      <c r="D62" s="12">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4">
+      <c r="B63" t="s">
+        <v>112</v>
+      </c>
+      <c r="C63" t="s">
+        <v>113</v>
+      </c>
+      <c r="D63" s="12">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4">
+      <c r="B64" t="s">
+        <v>114</v>
+      </c>
+      <c r="C64" t="s">
+        <v>115</v>
+      </c>
+      <c r="D64" s="12">
+        <v>46125</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D42" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:D43" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1782,107 +1926,107 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:1" ht="23.5">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="14" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="14" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="14" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="23.5">
+      <c r="A7" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="15"/>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" s="16" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" s="16" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" s="16" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="15" t="s">
+    <row r="12" spans="1:1">
+      <c r="A12" s="16" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="15" t="s">
+    <row r="14" spans="1:1" ht="23.5">
+      <c r="A14" s="13" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" s="15"/>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" s="15" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="15" t="s">
+    <row r="17" spans="1:1">
+      <c r="A17" s="15" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="23.5">
-      <c r="A7" s="14" t="s">
+    <row r="18" spans="1:1">
+      <c r="A18" s="15" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="16"/>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" s="17" t="s">
+    <row r="19" spans="1:1">
+      <c r="A19" s="15" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="17" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" s="15" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="17" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" s="15" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="12" spans="1:1">
-      <c r="A12" s="17" t="s">
+    <row r="23" spans="1:1" ht="23.5">
+      <c r="A23" s="13" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="23.5">
-      <c r="A14" s="14" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1">
-      <c r="A15" s="16"/>
-    </row>
-    <row r="16" spans="1:1">
-      <c r="A16" s="16" t="s">
+    <row r="24" spans="1:1">
+      <c r="A24" s="15"/>
+    </row>
+    <row r="25" spans="1:1">
+      <c r="A25" s="15" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
-      <c r="A17" s="16" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" s="15" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1">
-      <c r="A18" s="16" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1">
-      <c r="A19" s="16" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1">
-      <c r="A20" s="16" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" s="16" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" ht="23.5">
-      <c r="A23" s="14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1">
-      <c r="A24" s="16"/>
-    </row>
-    <row r="25" spans="1:1">
-      <c r="A25" s="16" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1">
-      <c r="A26" s="16" t="s">
-        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1896,8 +2040,8 @@
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="2" spans="1:1" ht="17.5">
-      <c r="A2" s="18" t="s">
-        <v>107</v>
+      <c r="A2" s="17" t="s">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Unified Next.js app: merge STRIQ SPA and garn-katalog
</commit_message>
<xml_diff>
--- a/STRIQ_ideer.xlsx
+++ b/STRIQ_ideer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\AI_projects\maskerummet\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDDA6467-8958-408C-BB65-55E7DF718A70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB0B46D8-A4A9-4C45-9E09-9B65A75FA4DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10650" yWindow="2850" windowWidth="16635" windowHeight="10605" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="STRIQ Ideer" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="172">
   <si>
     <t>Kategori</t>
   </si>
@@ -657,9 +657,6 @@
     <t>maskerummet.dk/#ideer</t>
   </si>
   <si>
-    <t>Se billede i link</t>
-  </si>
-  <si>
     <t>https://permin.dk/strik/opskrifter/bypermin-opskrifter/bella-opskrifter/stribet-raglansweater-med-martha-se5</t>
   </si>
   <si>
@@ -676,9 +673,6 @@
   </si>
   <si>
     <t>Bruges som case til substitution</t>
-  </si>
-  <si>
-    <t>substitution</t>
   </si>
   <si>
     <t xml:space="preserve">Case fra holland </t>
@@ -834,12 +828,72 @@
   <si>
     <t>Michele som partner</t>
   </si>
+  <si>
+    <t>dele færdige projekter med hinanden (uden at opskriften vises)</t>
+  </si>
+  <si>
+    <t>mulighed for flere fotos ved hvert færdigt projekt</t>
+  </si>
+  <si>
+    <t>Hvordan skaffer jeg sponsorer til sponsoreret content. Og hvordan ønsker jeg dette vist</t>
+  </si>
+  <si>
+    <t>AI farveanalyse af mit garn - hvordan kan dette løses/være interessant</t>
+  </si>
+  <si>
+    <t>Mønstre</t>
+  </si>
+  <si>
+    <t>Links til gratis mønstre hvor man kan få det vist med andet garn/farve. Første 2 visninger gratis. Herefter betaling</t>
+  </si>
+  <si>
+    <t>Model, hvor du kan se dig selv med en trøje på</t>
+  </si>
+  <si>
+    <t>Få lavet en opskrift baseret på et foto (ophavsret?)</t>
+  </si>
+  <si>
+    <t>Mønstre der ligger tilgængelige for alle, hvor man som medlem kan få den vist i andre farver</t>
+  </si>
+  <si>
+    <t>Er problemer med at gemme en opskrift eller billeder fra andre i et lukket system?</t>
+  </si>
+  <si>
+    <t>Undersøge GDPR</t>
+  </si>
+  <si>
+    <t>Links til podcasts og strikkebøger</t>
+  </si>
+  <si>
+    <t>links til garnfestivaler - og events. Kalender</t>
+  </si>
+  <si>
+    <t>Lækkert design</t>
+  </si>
+  <si>
+    <t>skal det også indbefatte hækling - hvad vil det kræve</t>
+  </si>
+  <si>
+    <t>mulighed for at sortere garnets visning på forsiden som man ønsker (default opsætning gemmes)</t>
+  </si>
+  <si>
+    <t>tilføje Lang yarns Baby alpaca til garn-kataloget</t>
+  </si>
+  <si>
+    <t>Tilføje aktuelle billigste pris til garn-kataloget (hvordan gør jeg det)</t>
+  </si>
+  <si>
+    <t>Vesterby Crea har et babyalpaka jeg ønsker at matche. Det er fra LangYarns</t>
+  </si>
+  <si>
+    <t>Jeg ønsker at strikke Mary baby plaid i det lækreste garn billigst muligt. Hvordan gør jeg det</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -965,6 +1019,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -987,37 +1056,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE8F5E9"/>
+        <fgColor rgb="FFE2D1F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE3F2FD"/>
+        <fgColor rgb="FFF8CBCB"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF3E0"/>
+        <fgColor rgb="FFBDD7EE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3E5F5"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE0F7FA"/>
+        <fgColor rgb="FFFCE4D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFBE9E7"/>
+        <fgColor rgb="FFD5F5F5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1041,7 +1110,7 @@
         <color rgb="FFD0C8BA"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE0E0E0"/>
+        <color rgb="FFD0D0D0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1053,10 +1122,10 @@
         <color rgb="FFD0C8BA"/>
       </right>
       <top style="thin">
-        <color rgb="FFE0E0E0"/>
+        <color rgb="FFD0D0D0"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE0E0E0"/>
+        <color rgb="FFD0D0D0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1064,10 +1133,10 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FFE0E0E0"/>
+        <color rgb="FFD0D0D0"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFE0E0E0"/>
+        <color rgb="FFD0D0D0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1075,7 +1144,7 @@
       <left/>
       <right/>
       <top style="thin">
-        <color rgb="FFE0E0E0"/>
+        <color rgb="FFD0D0D0"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -1085,9 +1154,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1102,140 +1170,134 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="6" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="18" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="7" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="6" fillId="8" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="8" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="18" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="7" fillId="9" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="18" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="9" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1730,798 +1792,958 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D64"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:D81"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="64.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="80.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.5703125" customWidth="1"/>
+    <col min="2" max="2" width="85" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="103.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="12" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4">
-      <c r="A2" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="11">
+      <c r="A2" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="16">
         <v>46101</v>
       </c>
     </row>
     <row r="3" spans="1:4">
-      <c r="A3" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="11">
+      <c r="A3" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="16">
         <v>46101</v>
       </c>
     </row>
     <row r="4" spans="1:4">
-      <c r="A4" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="13" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="15">
-        <v>46104</v>
+      <c r="A4" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="16">
+        <v>46101</v>
       </c>
     </row>
     <row r="5" spans="1:4">
-      <c r="A5" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>115</v>
-      </c>
-      <c r="D5" s="15">
+      <c r="A5" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="C5" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="D5" s="16">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>165</v>
+      </c>
+      <c r="C6" s="18"/>
+      <c r="D6" s="19"/>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="22">
         <v>46101</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="15">
-        <v>46104</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" s="15">
-        <v>46107</v>
-      </c>
-    </row>
     <row r="8" spans="1:4">
-      <c r="A8" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>117</v>
-      </c>
-      <c r="D8" s="15">
-        <v>46125</v>
+      <c r="A8" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>118</v>
+      </c>
+      <c r="D8" s="22">
+        <v>46101</v>
       </c>
     </row>
     <row r="9" spans="1:4">
-      <c r="A9" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" s="15">
-        <v>46104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="25">
-      <c r="A10" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D10" s="15">
-        <v>46111</v>
+      <c r="A9" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B9" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="22">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="22">
+        <v>46101</v>
       </c>
     </row>
     <row r="11" spans="1:4">
-      <c r="A11" s="16" t="s">
-        <v>4</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="D11" s="15">
-        <v>46122</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="17" customHeight="1">
+      <c r="A11" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="21"/>
+      <c r="D11" s="22">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="17.100000000000001" customHeight="1">
       <c r="A12" s="20" t="s">
-        <v>121</v>
+        <v>52</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>66</v>
+        <v>147</v>
       </c>
       <c r="C12" s="18"/>
-      <c r="D12" s="19">
-        <v>46120</v>
-      </c>
+      <c r="D12" s="19"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C13" s="18"/>
+      <c r="D13" s="19"/>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="C14" s="18"/>
+      <c r="D14" s="19"/>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="C15" s="18"/>
+      <c r="D15" s="19"/>
+    </row>
+    <row r="16" spans="1:4" ht="25.5">
+      <c r="A16" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="17" t="s">
+      <c r="B16" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C16" s="15"/>
+      <c r="D16" s="16">
+        <v>46120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="B17" s="14" t="s">
         <v>67</v>
       </c>
-      <c r="C13" s="18"/>
-      <c r="D13" s="19">
+      <c r="C17" s="15"/>
+      <c r="D17" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="20" t="s">
+    <row r="18" spans="1:4">
+      <c r="A18" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B18" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="19">
+      <c r="C18" s="15"/>
+      <c r="D18" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="20" t="s">
+    <row r="19" spans="1:4">
+      <c r="A19" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B15" s="17" t="s">
+      <c r="B19" s="14" t="s">
         <v>69</v>
       </c>
-      <c r="C15" s="18"/>
-      <c r="D15" s="19">
+      <c r="C19" s="15"/>
+      <c r="D19" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="20" t="s">
+    <row r="20" spans="1:4">
+      <c r="A20" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B16" s="17" t="s">
+      <c r="B20" s="14" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C20" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="19">
+      <c r="D20" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="20" t="s">
+    <row r="21" spans="1:4">
+      <c r="A21" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B17" s="17" t="s">
+      <c r="B21" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="C17" s="18" t="s">
+      <c r="C21" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D21" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" s="20" t="s">
+    <row r="22" spans="1:4">
+      <c r="A22" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B22" s="14" t="s">
         <v>75</v>
       </c>
-      <c r="C18" s="18" t="s">
+      <c r="C22" s="15" t="s">
         <v>74</v>
       </c>
-      <c r="D18" s="19">
+      <c r="D22" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="20" t="s">
+    <row r="23" spans="1:4">
+      <c r="A23" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B19" s="17" t="s">
+      <c r="B23" s="14" t="s">
         <v>76</v>
       </c>
-      <c r="C19" s="18" t="s">
+      <c r="C23" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D23" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="26">
-      <c r="A20" s="20" t="s">
+    <row r="24" spans="1:4">
+      <c r="A24" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B20" s="17" t="s">
+      <c r="B24" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="C20" s="18"/>
-      <c r="D20" s="19">
+      <c r="C24" s="15"/>
+      <c r="D24" s="16">
         <v>46120</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="25">
-      <c r="A21" s="20" t="s">
+    <row r="25" spans="1:4" ht="25.5">
+      <c r="A25" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B25" s="14" t="s">
         <v>100</v>
       </c>
-      <c r="C21" s="18" t="s">
+      <c r="C25" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D25" s="16">
         <v>46121</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="65">
-      <c r="A22" s="20" t="s">
+    <row r="26" spans="1:4" ht="51">
+      <c r="A26" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B22" s="17" t="s">
+      <c r="B26" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="C22" s="18"/>
-      <c r="D22" s="19">
+      <c r="C26" s="15"/>
+      <c r="D26" s="16">
         <v>46125</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="37.5">
-      <c r="A23" s="20" t="s">
+    <row r="27" spans="1:4" ht="38.25">
+      <c r="A27" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B27" s="14" t="s">
         <v>105</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C27" s="15" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D27" s="16">
         <v>46125</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
-      <c r="A24" s="20" t="s">
+    <row r="28" spans="1:4">
+      <c r="A28" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B24" s="17" t="s">
+      <c r="B28" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C28" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D28" s="16">
         <v>46125</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="25">
-      <c r="A25" s="20" t="s">
+    <row r="29" spans="1:4" ht="25.5">
+      <c r="A29" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B25" s="17" t="s">
+      <c r="B29" s="14" t="s">
         <v>109</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C29" s="15" t="s">
         <v>110</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D29" s="16">
         <v>46125</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" s="20" t="s">
+    <row r="30" spans="1:4">
+      <c r="A30" s="27" t="s">
         <v>121</v>
       </c>
-      <c r="B26" s="17" t="s">
+      <c r="B30" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C30" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D30" s="16">
         <v>46125</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" s="22" t="s">
-        <v>17</v>
-      </c>
-      <c r="D27" s="23">
+    <row r="31" spans="1:4">
+      <c r="A31" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="B31" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="18"/>
+      <c r="D31" s="19"/>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="C32" s="18"/>
+      <c r="D32" s="19"/>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B33" s="29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33" s="30" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="31">
         <v>46101</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
-      <c r="A28" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="C28" s="22"/>
-      <c r="D28" s="23">
+    <row r="34" spans="1:4">
+      <c r="A34" s="28" t="s">
+        <v>4</v>
+      </c>
+      <c r="B34" s="29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C34" s="30"/>
+      <c r="D34" s="31">
         <v>46101</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="A29" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>19</v>
-      </c>
-      <c r="C29" s="22" t="s">
-        <v>20</v>
-      </c>
-      <c r="D29" s="23">
+    <row r="35" spans="1:4">
+      <c r="A35" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D35" s="16">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
+      <c r="A36" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B36" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="D36" s="16">
         <v>46101</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="37.5">
-      <c r="A30" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="C30" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="D30" s="23">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>25</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D31" s="23">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
-      <c r="A32" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>28</v>
-      </c>
-      <c r="D32" s="23">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="25">
-      <c r="A33" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B33" s="21" t="s">
-        <v>29</v>
-      </c>
-      <c r="C33" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="D33" s="23">
+    <row r="37" spans="1:4">
+      <c r="A37" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B37" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="16">
         <v>46104</v>
       </c>
     </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B34" s="21" t="s">
-        <v>58</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>59</v>
-      </c>
-      <c r="D34" s="23">
+    <row r="38" spans="1:4">
+      <c r="A38" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="16">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>116</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="D39" s="16">
+        <v>46125</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B40" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D40" s="16">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="25.5">
+      <c r="A41" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D41" s="16">
         <v>46111</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="25">
-      <c r="A35" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B35" s="21" t="s">
-        <v>60</v>
-      </c>
-      <c r="C35" s="22" t="s">
-        <v>120</v>
-      </c>
-      <c r="D35" s="23">
-        <v>46112</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>64</v>
-      </c>
-      <c r="C36" s="22" t="s">
-        <v>65</v>
-      </c>
-      <c r="D36" s="23">
-        <v>46116</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B37" s="25" t="s">
-        <v>36</v>
-      </c>
-      <c r="C37" s="26" t="s">
-        <v>37</v>
-      </c>
-      <c r="D37" s="27">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4">
-      <c r="A38" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B38" s="25" t="s">
-        <v>38</v>
-      </c>
-      <c r="C38" s="26"/>
-      <c r="D38" s="27">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B39" s="25" t="s">
-        <v>39</v>
-      </c>
-      <c r="C39" s="26"/>
-      <c r="D39" s="27">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="28" t="s">
-        <v>35</v>
-      </c>
-      <c r="B40" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="C40" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="D40" s="27">
-        <v>46125</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41" s="29" t="s">
-        <v>40</v>
-      </c>
-      <c r="C41" s="30" t="s">
-        <v>41</v>
-      </c>
-      <c r="D41" s="31">
-        <v>46101</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="32" t="s">
-        <v>43</v>
-      </c>
-      <c r="B42" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C42" s="30" t="s">
-        <v>45</v>
-      </c>
-      <c r="D42" s="31">
-        <v>46101</v>
+        <v>4</v>
+      </c>
+      <c r="B42" s="14" t="s">
+        <v>102</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" s="16">
+        <v>46122</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="32" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" s="17" t="s">
+        <v>153</v>
+      </c>
+      <c r="C43" s="18"/>
+      <c r="D43" s="19"/>
+    </row>
+    <row r="44" spans="1:4" ht="25.5">
+      <c r="A44" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B44" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C44" s="34" t="s">
+        <v>17</v>
+      </c>
+      <c r="D44" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="25.5">
+      <c r="A45" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B45" s="14" t="s">
+        <v>18</v>
+      </c>
+      <c r="C45" s="34"/>
+      <c r="D45" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="25.5">
+      <c r="A46" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B46" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C46" s="34" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="38.25">
+      <c r="A47" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C47" s="34" t="s">
+        <v>24</v>
+      </c>
+      <c r="D47" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="25.5">
+      <c r="A48" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C48" s="34" t="s">
+        <v>26</v>
+      </c>
+      <c r="D48" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="25.5">
+      <c r="A49" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="C49" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D49" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="25.5">
+      <c r="A50" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="C50" s="34" t="s">
+        <v>30</v>
+      </c>
+      <c r="D50" s="35">
+        <v>46104</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="25.5">
+      <c r="A51" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C51" s="34" t="s">
+        <v>59</v>
+      </c>
+      <c r="D51" s="35">
+        <v>46111</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="25.5">
+      <c r="A52" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B52" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C52" s="34" t="s">
+        <v>120</v>
+      </c>
+      <c r="D52" s="35">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="25.5">
+      <c r="A53" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="B53" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C53" s="34" t="s">
+        <v>65</v>
+      </c>
+      <c r="D53" s="35">
+        <v>46116</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="25.5">
+      <c r="A54" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B54" s="37" t="s">
+        <v>148</v>
+      </c>
+      <c r="C54" s="38"/>
+      <c r="D54" s="39"/>
+    </row>
+    <row r="55" spans="1:4" ht="25.5">
+      <c r="A55" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B55" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="C55" s="38"/>
+      <c r="D55" s="39"/>
+    </row>
+    <row r="56" spans="1:4" ht="25.5">
+      <c r="A56" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B56" s="40" t="s">
+        <v>156</v>
+      </c>
+      <c r="C56" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="D56" s="39"/>
+    </row>
+    <row r="57" spans="1:4" ht="25.5">
+      <c r="A57" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B57" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="C57" s="38"/>
+      <c r="D57" s="39"/>
+    </row>
+    <row r="58" spans="1:4" ht="25.5">
+      <c r="A58" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B58" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="C58" s="38"/>
+      <c r="D58" s="39"/>
+    </row>
+    <row r="59" spans="1:4" ht="25.5">
+      <c r="A59" s="36" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="40" t="s">
+        <v>163</v>
+      </c>
+      <c r="C59" s="38"/>
+      <c r="D59" s="39"/>
+    </row>
+    <row r="60" spans="1:4">
+      <c r="A60" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B43" s="29" t="s">
+      <c r="B60" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="C60" s="34" t="s">
+        <v>41</v>
+      </c>
+      <c r="D60" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B61" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="C61" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="D61" s="35">
+        <v>46101</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B62" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="C43" s="30" t="s">
+      <c r="C62" s="34" t="s">
         <v>119</v>
       </c>
-      <c r="D43" s="31">
+      <c r="D62" s="35">
         <v>46101</v>
       </c>
     </row>
-    <row r="44" spans="1:4">
-      <c r="A44" s="32" t="s">
+    <row r="63" spans="1:4">
+      <c r="A63" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B44" s="29" t="s">
+      <c r="B63" s="37" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="33" t="s">
+      <c r="C63" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="D44" s="34">
+      <c r="D63" s="43">
         <v>46101</v>
       </c>
     </row>
-    <row r="45" spans="1:4">
-      <c r="A45" s="32" t="s">
+    <row r="64" spans="1:4">
+      <c r="A64" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B45" s="29" t="s">
+      <c r="B64" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="C45" s="33" t="s">
+      <c r="C64" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="D45" s="34">
+      <c r="D64" s="43">
         <v>46101</v>
       </c>
     </row>
-    <row r="46" spans="1:4">
-      <c r="A46" s="32" t="s">
+    <row r="65" spans="1:4">
+      <c r="A65" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B46" s="29" t="s">
+      <c r="B65" s="37" t="s">
         <v>51</v>
       </c>
-      <c r="C46" s="33"/>
-      <c r="D46" s="34">
+      <c r="C65" s="42"/>
+      <c r="D65" s="43">
         <v>46101</v>
       </c>
     </row>
-    <row r="47" spans="1:4" ht="39.5">
-      <c r="A47" s="32" t="s">
+    <row r="66" spans="1:4" ht="39">
+      <c r="A66" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B47" s="29" t="s">
+      <c r="B66" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="C47" s="35" t="s">
+      <c r="C66" s="44" t="s">
         <v>78</v>
       </c>
-      <c r="D47" s="34">
+      <c r="D66" s="43">
         <v>46120</v>
       </c>
     </row>
-    <row r="48" spans="1:4">
-      <c r="A48" s="32" t="s">
+    <row r="67" spans="1:4">
+      <c r="A67" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B48" s="29" t="s">
+      <c r="B67" s="37" t="s">
         <v>61</v>
       </c>
-      <c r="C48" s="33"/>
-      <c r="D48" s="34">
+      <c r="C67" s="42"/>
+      <c r="D67" s="43">
         <v>46115</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="26.5">
-      <c r="A49" s="32" t="s">
+    <row r="68" spans="1:4" ht="26.25">
+      <c r="A68" s="41" t="s">
         <v>43</v>
       </c>
-      <c r="B49" s="29" t="s">
+      <c r="B68" s="37" t="s">
         <v>62</v>
       </c>
-      <c r="C49" s="35" t="s">
+      <c r="C68" s="44" t="s">
         <v>63</v>
       </c>
-      <c r="D49" s="34">
+      <c r="D68" s="43">
         <v>46115</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
-      <c r="A50" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="B50" s="36" t="s">
-        <v>21</v>
-      </c>
-      <c r="C50" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="D50" s="38">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4">
-      <c r="A51" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="B51" s="36" t="s">
-        <v>42</v>
-      </c>
-      <c r="C51" s="40" t="s">
-        <v>118</v>
-      </c>
-      <c r="D51" s="38">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4">
-      <c r="A52" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="B52" s="36" t="s">
-        <v>53</v>
-      </c>
-      <c r="C52" s="37" t="s">
-        <v>54</v>
-      </c>
-      <c r="D52" s="38">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4">
-      <c r="A53" s="39" t="s">
-        <v>52</v>
-      </c>
-      <c r="B53" s="36" t="s">
-        <v>55</v>
-      </c>
-      <c r="C53" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="D53" s="38">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4">
-      <c r="A54" s="44" t="s">
-        <v>52</v>
-      </c>
-      <c r="B54" s="41" t="s">
-        <v>57</v>
-      </c>
-      <c r="C54" s="42"/>
-      <c r="D54" s="43">
-        <v>46101</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4">
-      <c r="A55" s="45" t="s">
-        <v>15</v>
-      </c>
-      <c r="C55" s="46" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4">
-      <c r="A56" s="45" t="s">
-        <v>130</v>
-      </c>
-      <c r="B56" s="47" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4">
-      <c r="B57" s="47" t="s">
-        <v>150</v>
-      </c>
-      <c r="D57" s="1"/>
-    </row>
-    <row r="58" spans="1:4">
-      <c r="B58" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4">
-      <c r="D59" s="1"/>
-    </row>
-    <row r="60" spans="1:4">
-      <c r="B60" t="s">
-        <v>151</v>
-      </c>
-      <c r="D60" s="1"/>
-    </row>
-    <row r="61" spans="1:4">
-      <c r="D61" s="1"/>
-    </row>
-    <row r="62" spans="1:4">
-      <c r="B62" t="s">
-        <v>152</v>
-      </c>
-      <c r="D62" s="1"/>
-    </row>
-    <row r="63" spans="1:4">
-      <c r="B63" t="s">
-        <v>153</v>
-      </c>
-      <c r="D63" s="1"/>
-    </row>
-    <row r="64" spans="1:4">
-      <c r="D64" s="1"/>
+    <row r="69" spans="1:4">
+      <c r="A69" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B69" s="40" t="s">
+        <v>155</v>
+      </c>
+      <c r="C69" s="38"/>
+      <c r="D69" s="39"/>
+    </row>
+    <row r="70" spans="1:4">
+      <c r="A70" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B70" s="40" t="s">
+        <v>158</v>
+      </c>
+      <c r="C70" s="38"/>
+      <c r="D70" s="39"/>
+    </row>
+    <row r="71" spans="1:4">
+      <c r="A71" s="41" t="s">
+        <v>43</v>
+      </c>
+      <c r="B71" s="40" t="s">
+        <v>159</v>
+      </c>
+      <c r="C71" s="38"/>
+      <c r="D71" s="39"/>
+    </row>
+    <row r="72" spans="1:4">
+      <c r="A72" s="45" t="s">
+        <v>43</v>
+      </c>
+      <c r="B72" s="46" t="s">
+        <v>161</v>
+      </c>
+      <c r="C72" s="47" t="s">
+        <v>162</v>
+      </c>
+      <c r="D72" s="48"/>
+    </row>
+    <row r="75" spans="1:4">
+      <c r="B75" s="49" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="B76" s="49" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="B77" s="49" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4">
+      <c r="B78" s="49" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4">
+      <c r="B79" s="49" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="81" spans="2:2">
+      <c r="B81" s="49" t="s">
+        <v>171</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2531,21 +2753,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FA47D4B-83C2-466D-8C5F-39F7D7509B1A}">
   <dimension ref="A2:L38"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="11:11">
       <c r="K2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="30" spans="12:12">
       <c r="L30" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2557,239 +2779,248 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A91C483-40FF-4FC6-A098-31A923F60DF5}">
   <dimension ref="B1:I65"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="2:2">
       <c r="B1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="45" spans="2:9">
       <c r="B45" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="2:9">
       <c r="B46" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="48" spans="2:9">
-      <c r="B48" s="48" t="s">
+      <c r="B48" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
+      <c r="H48" s="8"/>
+      <c r="I48" s="8"/>
+    </row>
+    <row r="49" spans="2:9">
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+      <c r="I49" s="9"/>
+    </row>
+    <row r="50" spans="2:9">
+      <c r="B50" s="8" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="8"/>
+      <c r="H50" s="8"/>
+      <c r="I50" s="8"/>
+    </row>
+    <row r="51" spans="2:9">
+      <c r="B51" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="C48" s="48"/>
-      <c r="D48" s="48"/>
-      <c r="E48" s="48"/>
-      <c r="F48" s="48"/>
-      <c r="G48" s="48"/>
-      <c r="H48" s="48"/>
-      <c r="I48" s="48"/>
-    </row>
-    <row r="49" spans="2:9">
-      <c r="B49" s="49"/>
-      <c r="C49" s="49"/>
-      <c r="D49" s="49"/>
-      <c r="E49" s="49"/>
-      <c r="F49" s="49"/>
-      <c r="G49" s="49"/>
-      <c r="H49" s="49"/>
-      <c r="I49" s="49"/>
-    </row>
-    <row r="50" spans="2:9">
-      <c r="B50" s="48" t="s">
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+    </row>
+    <row r="52" spans="2:9">
+      <c r="B52" s="11" t="s">
         <v>133</v>
       </c>
-      <c r="C50" s="48"/>
-      <c r="D50" s="48"/>
-      <c r="E50" s="48"/>
-      <c r="F50" s="48"/>
-      <c r="G50" s="48"/>
-      <c r="H50" s="48"/>
-      <c r="I50" s="48"/>
-    </row>
-    <row r="51" spans="2:9">
-      <c r="B51" s="50" t="s">
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="11"/>
+      <c r="F52" s="11"/>
+      <c r="G52" s="11"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
+    </row>
+    <row r="53" spans="2:9">
+      <c r="B53" s="11" t="s">
         <v>134</v>
       </c>
-      <c r="C51" s="50"/>
-      <c r="D51" s="50"/>
-      <c r="E51" s="50"/>
-      <c r="F51" s="50"/>
-      <c r="G51" s="50"/>
-      <c r="H51" s="50"/>
-      <c r="I51" s="50"/>
-    </row>
-    <row r="52" spans="2:9">
-      <c r="B52" s="51" t="s">
+      <c r="C53" s="11"/>
+      <c r="D53" s="11"/>
+      <c r="E53" s="11"/>
+      <c r="F53" s="11"/>
+      <c r="G53" s="11"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+    </row>
+    <row r="54" spans="2:9">
+      <c r="B54" s="11" t="s">
         <v>135</v>
       </c>
-      <c r="C52" s="51"/>
-      <c r="D52" s="51"/>
-      <c r="E52" s="51"/>
-      <c r="F52" s="51"/>
-      <c r="G52" s="51"/>
-      <c r="H52" s="51"/>
-      <c r="I52" s="51"/>
-    </row>
-    <row r="53" spans="2:9">
-      <c r="B53" s="51" t="s">
+      <c r="C54" s="11"/>
+      <c r="D54" s="11"/>
+      <c r="E54" s="11"/>
+      <c r="F54" s="11"/>
+      <c r="G54" s="11"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="11"/>
+    </row>
+    <row r="55" spans="2:9">
+      <c r="B55" s="11" t="s">
         <v>136</v>
       </c>
-      <c r="C53" s="51"/>
-      <c r="D53" s="51"/>
-      <c r="E53" s="51"/>
-      <c r="F53" s="51"/>
-      <c r="G53" s="51"/>
-      <c r="H53" s="51"/>
-      <c r="I53" s="51"/>
-    </row>
-    <row r="54" spans="2:9">
-      <c r="B54" s="51" t="s">
+      <c r="C55" s="11"/>
+      <c r="D55" s="11"/>
+      <c r="E55" s="11"/>
+      <c r="F55" s="11"/>
+      <c r="G55" s="11"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
+    </row>
+    <row r="56" spans="2:9">
+      <c r="B56" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="C54" s="51"/>
-      <c r="D54" s="51"/>
-      <c r="E54" s="51"/>
-      <c r="F54" s="51"/>
-      <c r="G54" s="51"/>
-      <c r="H54" s="51"/>
-      <c r="I54" s="51"/>
-    </row>
-    <row r="55" spans="2:9">
-      <c r="B55" s="51" t="s">
+      <c r="C56" s="11"/>
+      <c r="D56" s="11"/>
+      <c r="E56" s="11"/>
+      <c r="F56" s="11"/>
+      <c r="G56" s="11"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+    </row>
+    <row r="57" spans="2:9">
+      <c r="B57" s="7" t="s">
         <v>138</v>
       </c>
-      <c r="C55" s="51"/>
-      <c r="D55" s="51"/>
-      <c r="E55" s="51"/>
-      <c r="F55" s="51"/>
-      <c r="G55" s="51"/>
-      <c r="H55" s="51"/>
-      <c r="I55" s="51"/>
-    </row>
-    <row r="56" spans="2:9">
-      <c r="B56" s="51" t="s">
+      <c r="C57" s="7"/>
+      <c r="D57" s="7"/>
+      <c r="E57" s="7"/>
+      <c r="F57" s="7"/>
+      <c r="G57" s="7"/>
+      <c r="H57" s="7"/>
+      <c r="I57" s="7"/>
+    </row>
+    <row r="58" spans="2:9">
+      <c r="B58" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="C56" s="51"/>
-      <c r="D56" s="51"/>
-      <c r="E56" s="51"/>
-      <c r="F56" s="51"/>
-      <c r="G56" s="51"/>
-      <c r="H56" s="51"/>
-      <c r="I56" s="51"/>
-    </row>
-    <row r="57" spans="2:9">
-      <c r="B57" s="52" t="s">
+      <c r="C58" s="7"/>
+      <c r="D58" s="7"/>
+      <c r="E58" s="7"/>
+      <c r="F58" s="7"/>
+      <c r="G58" s="7"/>
+      <c r="H58" s="7"/>
+      <c r="I58" s="7"/>
+    </row>
+    <row r="59" spans="2:9">
+      <c r="B59" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="C57" s="52"/>
-      <c r="D57" s="52"/>
-      <c r="E57" s="52"/>
-      <c r="F57" s="52"/>
-      <c r="G57" s="52"/>
-      <c r="H57" s="52"/>
-      <c r="I57" s="52"/>
-    </row>
-    <row r="58" spans="2:9">
-      <c r="B58" s="52" t="s">
+      <c r="C59" s="7"/>
+      <c r="D59" s="7"/>
+      <c r="E59" s="7"/>
+      <c r="F59" s="7"/>
+      <c r="G59" s="7"/>
+      <c r="H59" s="7"/>
+      <c r="I59" s="7"/>
+    </row>
+    <row r="60" spans="2:9">
+      <c r="B60" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="C58" s="52"/>
-      <c r="D58" s="52"/>
-      <c r="E58" s="52"/>
-      <c r="F58" s="52"/>
-      <c r="G58" s="52"/>
-      <c r="H58" s="52"/>
-      <c r="I58" s="52"/>
-    </row>
-    <row r="59" spans="2:9">
-      <c r="B59" s="52" t="s">
+      <c r="C60" s="7"/>
+      <c r="D60" s="7"/>
+      <c r="E60" s="7"/>
+      <c r="F60" s="7"/>
+      <c r="G60" s="7"/>
+      <c r="H60" s="7"/>
+      <c r="I60" s="7"/>
+    </row>
+    <row r="61" spans="2:9">
+      <c r="B61" s="7" t="s">
         <v>142</v>
       </c>
-      <c r="C59" s="52"/>
-      <c r="D59" s="52"/>
-      <c r="E59" s="52"/>
-      <c r="F59" s="52"/>
-      <c r="G59" s="52"/>
-      <c r="H59" s="52"/>
-      <c r="I59" s="52"/>
-    </row>
-    <row r="60" spans="2:9">
-      <c r="B60" s="52" t="s">
+      <c r="C61" s="7"/>
+      <c r="D61" s="7"/>
+      <c r="E61" s="7"/>
+      <c r="F61" s="7"/>
+      <c r="G61" s="7"/>
+      <c r="H61" s="7"/>
+      <c r="I61" s="7"/>
+    </row>
+    <row r="62" spans="2:9">
+      <c r="B62" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="C60" s="52"/>
-      <c r="D60" s="52"/>
-      <c r="E60" s="52"/>
-      <c r="F60" s="52"/>
-      <c r="G60" s="52"/>
-      <c r="H60" s="52"/>
-      <c r="I60" s="52"/>
-    </row>
-    <row r="61" spans="2:9">
-      <c r="B61" s="52" t="s">
+      <c r="C62" s="7"/>
+      <c r="D62" s="7"/>
+      <c r="E62" s="7"/>
+      <c r="F62" s="7"/>
+      <c r="G62" s="7"/>
+      <c r="H62" s="7"/>
+      <c r="I62" s="7"/>
+    </row>
+    <row r="63" spans="2:9">
+      <c r="B63" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="C61" s="52"/>
-      <c r="D61" s="52"/>
-      <c r="E61" s="52"/>
-      <c r="F61" s="52"/>
-      <c r="G61" s="52"/>
-      <c r="H61" s="52"/>
-      <c r="I61" s="52"/>
-    </row>
-    <row r="62" spans="2:9">
-      <c r="B62" s="52" t="s">
+      <c r="C63" s="7"/>
+      <c r="D63" s="7"/>
+      <c r="E63" s="7"/>
+      <c r="F63" s="7"/>
+      <c r="G63" s="7"/>
+      <c r="H63" s="7"/>
+      <c r="I63" s="7"/>
+    </row>
+    <row r="64" spans="2:9">
+      <c r="B64" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C62" s="52"/>
-      <c r="D62" s="52"/>
-      <c r="E62" s="52"/>
-      <c r="F62" s="52"/>
-      <c r="G62" s="52"/>
-      <c r="H62" s="52"/>
-      <c r="I62" s="52"/>
-    </row>
-    <row r="63" spans="2:9">
-      <c r="B63" s="52" t="s">
+      <c r="C64" s="7"/>
+      <c r="D64" s="7"/>
+      <c r="E64" s="7"/>
+      <c r="F64" s="7"/>
+      <c r="G64" s="7"/>
+      <c r="H64" s="7"/>
+      <c r="I64" s="7"/>
+    </row>
+    <row r="65" spans="2:9" ht="21.95" customHeight="1">
+      <c r="B65" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="C63" s="52"/>
-      <c r="D63" s="52"/>
-      <c r="E63" s="52"/>
-      <c r="F63" s="52"/>
-      <c r="G63" s="52"/>
-      <c r="H63" s="52"/>
-      <c r="I63" s="52"/>
-    </row>
-    <row r="64" spans="2:9">
-      <c r="B64" s="52" t="s">
-        <v>147</v>
-      </c>
-      <c r="C64" s="52"/>
-      <c r="D64" s="52"/>
-      <c r="E64" s="52"/>
-      <c r="F64" s="52"/>
-      <c r="G64" s="52"/>
-      <c r="H64" s="52"/>
-      <c r="I64" s="52"/>
-    </row>
-    <row r="65" spans="2:9" ht="22" customHeight="1">
-      <c r="B65" s="52" t="s">
-        <v>148</v>
-      </c>
-      <c r="C65" s="52"/>
-      <c r="D65" s="52"/>
-      <c r="E65" s="52"/>
-      <c r="F65" s="52"/>
-      <c r="G65" s="52"/>
-      <c r="H65" s="52"/>
-      <c r="I65" s="52"/>
+      <c r="C65" s="7"/>
+      <c r="D65" s="7"/>
+      <c r="E65" s="7"/>
+      <c r="F65" s="7"/>
+      <c r="G65" s="7"/>
+      <c r="H65" s="7"/>
+      <c r="I65" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B53:I53"/>
+    <mergeCell ref="B54:I54"/>
+    <mergeCell ref="B55:I55"/>
+    <mergeCell ref="B56:I56"/>
+    <mergeCell ref="B48:I48"/>
+    <mergeCell ref="B49:I49"/>
+    <mergeCell ref="B50:I50"/>
+    <mergeCell ref="B51:I51"/>
+    <mergeCell ref="B52:I52"/>
     <mergeCell ref="B63:I63"/>
     <mergeCell ref="B64:I64"/>
     <mergeCell ref="B65:I65"/>
@@ -2799,15 +3030,6 @@
     <mergeCell ref="B60:I60"/>
     <mergeCell ref="B61:I61"/>
     <mergeCell ref="B62:I62"/>
-    <mergeCell ref="B48:I48"/>
-    <mergeCell ref="B49:I49"/>
-    <mergeCell ref="B50:I50"/>
-    <mergeCell ref="B51:I51"/>
-    <mergeCell ref="B52:I52"/>
-    <mergeCell ref="B53:I53"/>
-    <mergeCell ref="B54:I54"/>
-    <mergeCell ref="B55:I55"/>
-    <mergeCell ref="B56:I56"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="B65" r:id="rId1" display="https://dk.mypz.nl/products/mypz-starlight-gold" xr:uid="{38639F60-8605-4A9D-82D3-BF3CA851C39F}"/>
@@ -2833,10 +3055,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F20B0B5D-FE18-403D-8A17-9DD1BE07C0C9}">
   <dimension ref="A2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="2" spans="1:1">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>122</v>
       </c>
     </row>
@@ -2848,109 +3070,109 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76A877B6-DA4E-4112-95A7-38B2DD01CB5F}">
   <dimension ref="A1:A26"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:1" ht="23.5">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:1" ht="23.25">
+      <c r="A1" s="1" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="23.5">
-      <c r="A7" s="2" t="s">
+    <row r="7" spans="1:1" ht="23.25">
+      <c r="A7" s="1" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="4"/>
+      <c r="A8" s="3"/>
     </row>
     <row r="9" spans="1:1">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="4" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="10" spans="1:1">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="4" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:1">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="4" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="12" spans="1:1">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="4" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="23.5">
-      <c r="A14" s="2" t="s">
+    <row r="14" spans="1:1" ht="23.25">
+      <c r="A14" s="1" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="15" spans="1:1">
-      <c r="A15" s="4"/>
+      <c r="A15" s="3"/>
     </row>
     <row r="16" spans="1:1">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="4" t="s">
+      <c r="A17" s="3" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="4" t="s">
+      <c r="A18" s="3" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="3" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="3" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="23.5">
-      <c r="A23" s="2" t="s">
+    <row r="23" spans="1:1" ht="23.25">
+      <c r="A23" s="1" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="4"/>
+      <c r="A24" s="3"/>
     </row>
     <row r="25" spans="1:1">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="3" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="26" spans="1:1">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="3" t="s">
         <v>97</v>
       </c>
     </row>
@@ -2962,10 +3184,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{195BDE92-4573-4352-B207-D116866D70A3}">
   <dimension ref="A2"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="1:1" ht="17.5">
-      <c r="A2" s="6" t="s">
+    <row r="2" spans="1:1" ht="17.25">
+      <c r="A2" s="5" t="s">
         <v>99</v>
       </c>
     </row>

</xml_diff>